<commit_message>
Revert project to Document Authoring (DA) configuration
Correct the project type from xwalk back to DA and remove the
Universal Editor artifacts that were added by mistake.

- Fix .migration/project.json to flat DA shape (type "da", lowercase
  org "adobedrago", contentHostUrl) and update fstab.yaml mountpoint
- Remove xwalk artifacts: root component-*.json, models/, and the
  per-block _<block>.json model files
- Drop build:json scripts and xwalk devDeps from package.json and
  plugin:xwalk/recommended from .eslintrc.js
- Revert field-hint comments from the container parsers and re-import
  all 3 pages so content is clean DA

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-insurance-hub.report.xlsx
+++ b/tools/importer/reports/import-insurance-hub.report.xlsx
@@ -52,7 +52,7 @@
     <t>insurance-hub</t>
   </si>
   <si>
-    <t>2026-07-09T16:31:59.124Z</t>
+    <t>2026-07-09T16:54:29.833Z</t>
   </si>
   <si>
     <t>Types of Insurance Coverage | State Farm® - State Farm®</t>
@@ -73,7 +73,7 @@
     <t>insurance-product</t>
   </si>
   <si>
-    <t>2026-07-09T14:45:53.991Z</t>
+    <t>2026-07-09T16:32:10.947Z</t>
   </si>
   <si>
     <t>Car Insurance | Free Auto Insurance Quote</t>
@@ -91,7 +91,7 @@
     <t>insurance/homeowners</t>
   </si>
   <si>
-    <t>2026-07-09T16:16:13.384Z</t>
+    <t>2026-07-09T16:32:20.743Z</t>
   </si>
   <si>
     <t>Homeowners Insurance: Get a free quote today</t>

</xml_diff>